<commit_message>
Replace notebooks with Python scripts and update pipeline
</commit_message>
<xml_diff>
--- a/src/data/liberacao_tecnicos_clientes.xlsx
+++ b/src/data/liberacao_tecnicos_clientes.xlsx
@@ -473,12 +473,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -500,17 +500,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -532,12 +532,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -702,17 +702,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -724,17 +724,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -820,17 +820,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -980,22 +980,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1108,27 +1108,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1315,12 +1315,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>liberado</t>
+          <t>bloqueado</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
     </row>
@@ -1401,22 +1401,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>bloqueado</t>
+          <t>liberado</t>
         </is>
       </c>
     </row>

</xml_diff>